<commit_message>
Parecer em página 2 dedicada (Excel e PDF)
O Parecer deixa de ocupar um pequeno espaço no fim da página 1 e passa a
ser uma folha A4 quase inteira, em branco, na página 2 — título PARECER,
campos Nome/Data não preenchidos e 27 linhas com borda inferior para
escrita manual. Página 1 continua fiel ao formulário oficial, agora
terminando na assinatura do avaliador (o pequeno bloco "Parecer" antigo,
que ficava colado ao rodapé do formulário, foi removido).

No Excel, isso exigiu mover a linha de assinatura (A51->A46), adicionar
quebra de página manual após a linha 46 e um scale de 96% para garantir
exatamente 2 páginas de impressão (validado via Excel COM real, não só
estrutura XML). No PDF, pdfTemplate.js agora monta duas páginas A4
separadas e pdfExport.js as renderiza cada uma em sua própria página do
PDF.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/teste-pratico-motoristas.xlsx
+++ b/templates/teste-pratico-motoristas.xlsx
@@ -15,6 +15,9 @@
   <sheets>
     <sheet name="ATUALIZADO MARÇO-2025" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ATUALIZADO MARÇO-2025'!$A$1:$H$77</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1156,7 +1159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1475,6 +1478,15 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1810,7 +1822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93870B26-7C85-41EC-983A-E51F9F679233}">
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.5546875" style="1" customWidth="1"/>
@@ -2390,362 +2402,324 @@
       <c r="G45" s="43"/>
       <c r="H45" s="43"/>
     </row>
-    <row r="46" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="43"/>
-      <c r="B46" s="43"/>
-      <c r="C46" s="43"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="43"/>
-    </row>
-    <row r="47" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="36"/>
-      <c r="B47" s="37"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="37"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="38"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A48" s="32"/>
-      <c r="B48" s="67" t="s">
-        <v>54</v>
-      </c>
-      <c r="C48" s="68"/>
-      <c r="D48" s="68"/>
-      <c r="E48" s="68"/>
-      <c r="F48" s="68"/>
-      <c r="G48" s="69"/>
-      <c r="H48" s="33"/>
-    </row>
-    <row r="49" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="32"/>
-      <c r="B49" s="70"/>
-      <c r="C49" s="71"/>
-      <c r="D49" s="71"/>
-      <c r="E49" s="71"/>
-      <c r="F49" s="71"/>
-      <c r="G49" s="72"/>
-      <c r="H49" s="33"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="32"/>
-      <c r="B50" s="43"/>
-      <c r="C50" s="43"/>
-      <c r="D50" s="43"/>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="33"/>
-    </row>
-    <row r="51" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="73" t="s">
+    <row r="46" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="73" t="s">
         <v>53</v>
       </c>
-      <c r="B51" s="74"/>
-      <c r="C51" s="74"/>
-      <c r="D51" s="74"/>
-      <c r="E51" s="74"/>
-      <c r="F51" s="74"/>
-      <c r="G51" s="74"/>
-      <c r="H51" s="75"/>
-    </row>
-    <row r="52" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="56"/>
-      <c r="B52" s="57"/>
-      <c r="C52" s="57"/>
-      <c r="D52" s="57"/>
-      <c r="E52" s="57"/>
-      <c r="F52" s="57"/>
-      <c r="G52" s="57"/>
-      <c r="H52" s="58"/>
-    </row>
-    <row r="53" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="29"/>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
-      <c r="F53" s="30"/>
-      <c r="G53" s="30"/>
-      <c r="H53" s="31"/>
-    </row>
-    <row r="54" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="29"/>
-      <c r="B54" s="30"/>
-      <c r="C54" s="30"/>
-      <c r="D54" s="30"/>
-      <c r="E54" s="30"/>
-      <c r="F54" s="30"/>
-      <c r="G54" s="30"/>
-      <c r="H54" s="31"/>
-    </row>
-    <row r="55" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="29"/>
-      <c r="B55" s="30"/>
-      <c r="C55" s="30"/>
-      <c r="D55" s="30"/>
-      <c r="E55" s="30"/>
-      <c r="F55" s="30"/>
-      <c r="G55" s="30"/>
-      <c r="H55" s="31"/>
-    </row>
-    <row r="56" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="29"/>
-      <c r="B56" s="30"/>
-      <c r="C56" s="30"/>
-      <c r="D56" s="30"/>
-      <c r="E56" s="30"/>
-      <c r="F56" s="30"/>
-      <c r="G56" s="30"/>
-      <c r="H56" s="31"/>
-    </row>
-    <row r="57" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="2"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
-      <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="4"/>
-    </row>
-    <row r="58" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="2"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="4"/>
-    </row>
-    <row r="59" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="2"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-      <c r="G59" s="3"/>
-      <c r="H59" s="4"/>
-    </row>
-    <row r="60" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="2"/>
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="3"/>
-      <c r="G60" s="3"/>
-      <c r="H60" s="4"/>
-    </row>
-    <row r="61" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="2"/>
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
-      <c r="D61" s="3"/>
-      <c r="E61" s="3"/>
-      <c r="F61" s="3"/>
-      <c r="G61" s="3"/>
-      <c r="H61" s="4"/>
-    </row>
-    <row r="62" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="2"/>
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
-      <c r="F62" s="3"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="4"/>
-    </row>
-    <row r="63" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="2"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="E63" s="3"/>
-      <c r="F63" s="3"/>
-      <c r="G63" s="3"/>
-      <c r="H63" s="4"/>
-    </row>
-    <row r="64" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="2"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
-      <c r="G64" s="3"/>
-      <c r="H64" s="4"/>
-    </row>
-    <row r="65" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="2"/>
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="D65" s="3"/>
-      <c r="E65" s="3"/>
-      <c r="F65" s="3"/>
-      <c r="G65" s="3"/>
-      <c r="H65" s="4"/>
-    </row>
-    <row r="66" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="2"/>
-      <c r="B66" s="3"/>
-      <c r="C66" s="3"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="3"/>
-      <c r="F66" s="3"/>
-      <c r="G66" s="3"/>
-      <c r="H66" s="4"/>
-    </row>
-    <row r="67" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="2"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="3"/>
-      <c r="H67" s="4"/>
-    </row>
-    <row r="68" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="2"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-      <c r="G68" s="3"/>
-      <c r="H68" s="4"/>
-    </row>
-    <row r="69" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="2"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="3"/>
-      <c r="H69" s="4"/>
-    </row>
-    <row r="70" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="2"/>
-      <c r="B70" s="3"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="3"/>
-      <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="3"/>
-      <c r="H70" s="4"/>
-    </row>
-    <row r="71" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="2"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="3"/>
-      <c r="H71" s="4"/>
-    </row>
-    <row r="72" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="2"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="4"/>
-    </row>
-    <row r="73" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="2"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="4"/>
-    </row>
-    <row r="74" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="2"/>
-      <c r="B74" s="3"/>
-      <c r="C74" s="3"/>
-      <c r="D74" s="3"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="4"/>
-    </row>
-    <row r="75" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="2"/>
-      <c r="B75" s="3"/>
-      <c r="C75" s="3"/>
-      <c r="D75" s="3"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
-      <c r="G75" s="3"/>
-      <c r="H75" s="4"/>
-    </row>
-    <row r="76" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="2"/>
-      <c r="B76" s="3"/>
-      <c r="C76" s="3"/>
-      <c r="D76" s="3"/>
-      <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
-      <c r="G76" s="3"/>
-      <c r="H76" s="4"/>
-    </row>
-    <row r="77" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="2"/>
-      <c r="B77" s="3"/>
-      <c r="C77" s="3"/>
-      <c r="D77" s="3"/>
-      <c r="E77" s="3"/>
-      <c r="F77" s="3"/>
-      <c r="G77" s="3"/>
-      <c r="H77" s="4"/>
-    </row>
-    <row r="78" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="2"/>
-      <c r="B78" s="3"/>
-      <c r="C78" s="3"/>
-      <c r="D78" s="3"/>
-      <c r="E78" s="3"/>
-      <c r="F78" s="3"/>
-      <c r="G78" s="3"/>
-      <c r="H78" s="4"/>
-    </row>
-    <row r="79" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="2"/>
-      <c r="B79" s="3"/>
-      <c r="C79" s="3"/>
-      <c r="D79" s="3"/>
-      <c r="E79" s="3"/>
-      <c r="F79" s="3"/>
-      <c r="G79" s="3"/>
-      <c r="H79" s="4"/>
-    </row>
-    <row r="80" spans="1:8" ht="21.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="44"/>
-      <c r="B80" s="45"/>
-      <c r="C80" s="45"/>
-      <c r="D80" s="45"/>
-      <c r="E80" s="45"/>
-      <c r="F80" s="45"/>
-      <c r="G80" s="45"/>
-      <c r="H80" s="46"/>
+      <c r="B46" s="74"/>
+      <c r="C46" s="74"/>
+      <c r="D46" s="74"/>
+      <c r="E46" s="74"/>
+      <c r="F46" s="74"/>
+      <c r="G46" s="74"/>
+      <c r="H46" s="75"/>
+    </row>
+    <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARECER</t>
+        </is>
+      </c>
+      <c r="B47" s="107"/>
+      <c r="C47" s="107"/>
+      <c r="D47" s="107"/>
+      <c r="E47" s="107"/>
+      <c r="F47" s="107"/>
+      <c r="G47" s="107"/>
+      <c r="H47" s="107"/>
+    </row>
+    <row r="48" spans="1:8" ht="10" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome:</t>
+        </is>
+      </c>
+      <c r="B49" s="108"/>
+      <c r="C49" s="109"/>
+      <c r="D49" s="109"/>
+      <c r="E49" s="109"/>
+      <c r="F49" s="109"/>
+      <c r="G49" s="108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data:</t>
+        </is>
+      </c>
+      <c r="H49" s="109"/>
+    </row>
+    <row r="50" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="109"/>
+      <c r="B51" s="109"/>
+      <c r="C51" s="109"/>
+      <c r="D51" s="109"/>
+      <c r="E51" s="109"/>
+      <c r="F51" s="109"/>
+      <c r="G51" s="109"/>
+      <c r="H51" s="109"/>
+    </row>
+    <row r="52" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="109"/>
+      <c r="B52" s="109"/>
+      <c r="C52" s="109"/>
+      <c r="D52" s="109"/>
+      <c r="E52" s="109"/>
+      <c r="F52" s="109"/>
+      <c r="G52" s="109"/>
+      <c r="H52" s="109"/>
+    </row>
+    <row r="53" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="109"/>
+      <c r="B53" s="109"/>
+      <c r="C53" s="109"/>
+      <c r="D53" s="109"/>
+      <c r="E53" s="109"/>
+      <c r="F53" s="109"/>
+      <c r="G53" s="109"/>
+      <c r="H53" s="109"/>
+    </row>
+    <row r="54" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="109"/>
+      <c r="B54" s="109"/>
+      <c r="C54" s="109"/>
+      <c r="D54" s="109"/>
+      <c r="E54" s="109"/>
+      <c r="F54" s="109"/>
+      <c r="G54" s="109"/>
+      <c r="H54" s="109"/>
+    </row>
+    <row r="55" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="109"/>
+      <c r="B55" s="109"/>
+      <c r="C55" s="109"/>
+      <c r="D55" s="109"/>
+      <c r="E55" s="109"/>
+      <c r="F55" s="109"/>
+      <c r="G55" s="109"/>
+      <c r="H55" s="109"/>
+    </row>
+    <row r="56" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="109"/>
+      <c r="B56" s="109"/>
+      <c r="C56" s="109"/>
+      <c r="D56" s="109"/>
+      <c r="E56" s="109"/>
+      <c r="F56" s="109"/>
+      <c r="G56" s="109"/>
+      <c r="H56" s="109"/>
+    </row>
+    <row r="57" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="109"/>
+      <c r="B57" s="109"/>
+      <c r="C57" s="109"/>
+      <c r="D57" s="109"/>
+      <c r="E57" s="109"/>
+      <c r="F57" s="109"/>
+      <c r="G57" s="109"/>
+      <c r="H57" s="109"/>
+    </row>
+    <row r="58" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="109"/>
+      <c r="B58" s="109"/>
+      <c r="C58" s="109"/>
+      <c r="D58" s="109"/>
+      <c r="E58" s="109"/>
+      <c r="F58" s="109"/>
+      <c r="G58" s="109"/>
+      <c r="H58" s="109"/>
+    </row>
+    <row r="59" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="109"/>
+      <c r="B59" s="109"/>
+      <c r="C59" s="109"/>
+      <c r="D59" s="109"/>
+      <c r="E59" s="109"/>
+      <c r="F59" s="109"/>
+      <c r="G59" s="109"/>
+      <c r="H59" s="109"/>
+    </row>
+    <row r="60" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="109"/>
+      <c r="B60" s="109"/>
+      <c r="C60" s="109"/>
+      <c r="D60" s="109"/>
+      <c r="E60" s="109"/>
+      <c r="F60" s="109"/>
+      <c r="G60" s="109"/>
+      <c r="H60" s="109"/>
+    </row>
+    <row r="61" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="109"/>
+      <c r="B61" s="109"/>
+      <c r="C61" s="109"/>
+      <c r="D61" s="109"/>
+      <c r="E61" s="109"/>
+      <c r="F61" s="109"/>
+      <c r="G61" s="109"/>
+      <c r="H61" s="109"/>
+    </row>
+    <row r="62" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="109"/>
+      <c r="B62" s="109"/>
+      <c r="C62" s="109"/>
+      <c r="D62" s="109"/>
+      <c r="E62" s="109"/>
+      <c r="F62" s="109"/>
+      <c r="G62" s="109"/>
+      <c r="H62" s="109"/>
+    </row>
+    <row r="63" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="109"/>
+      <c r="B63" s="109"/>
+      <c r="C63" s="109"/>
+      <c r="D63" s="109"/>
+      <c r="E63" s="109"/>
+      <c r="F63" s="109"/>
+      <c r="G63" s="109"/>
+      <c r="H63" s="109"/>
+    </row>
+    <row r="64" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="109"/>
+      <c r="B64" s="109"/>
+      <c r="C64" s="109"/>
+      <c r="D64" s="109"/>
+      <c r="E64" s="109"/>
+      <c r="F64" s="109"/>
+      <c r="G64" s="109"/>
+      <c r="H64" s="109"/>
+    </row>
+    <row r="65" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="109"/>
+      <c r="B65" s="109"/>
+      <c r="C65" s="109"/>
+      <c r="D65" s="109"/>
+      <c r="E65" s="109"/>
+      <c r="F65" s="109"/>
+      <c r="G65" s="109"/>
+      <c r="H65" s="109"/>
+    </row>
+    <row r="66" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="109"/>
+      <c r="B66" s="109"/>
+      <c r="C66" s="109"/>
+      <c r="D66" s="109"/>
+      <c r="E66" s="109"/>
+      <c r="F66" s="109"/>
+      <c r="G66" s="109"/>
+      <c r="H66" s="109"/>
+    </row>
+    <row r="67" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="109"/>
+      <c r="B67" s="109"/>
+      <c r="C67" s="109"/>
+      <c r="D67" s="109"/>
+      <c r="E67" s="109"/>
+      <c r="F67" s="109"/>
+      <c r="G67" s="109"/>
+      <c r="H67" s="109"/>
+    </row>
+    <row r="68" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="109"/>
+      <c r="B68" s="109"/>
+      <c r="C68" s="109"/>
+      <c r="D68" s="109"/>
+      <c r="E68" s="109"/>
+      <c r="F68" s="109"/>
+      <c r="G68" s="109"/>
+      <c r="H68" s="109"/>
+    </row>
+    <row r="69" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="109"/>
+      <c r="B69" s="109"/>
+      <c r="C69" s="109"/>
+      <c r="D69" s="109"/>
+      <c r="E69" s="109"/>
+      <c r="F69" s="109"/>
+      <c r="G69" s="109"/>
+      <c r="H69" s="109"/>
+    </row>
+    <row r="70" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="109"/>
+      <c r="B70" s="109"/>
+      <c r="C70" s="109"/>
+      <c r="D70" s="109"/>
+      <c r="E70" s="109"/>
+      <c r="F70" s="109"/>
+      <c r="G70" s="109"/>
+      <c r="H70" s="109"/>
+    </row>
+    <row r="71" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="109"/>
+      <c r="B71" s="109"/>
+      <c r="C71" s="109"/>
+      <c r="D71" s="109"/>
+      <c r="E71" s="109"/>
+      <c r="F71" s="109"/>
+      <c r="G71" s="109"/>
+      <c r="H71" s="109"/>
+    </row>
+    <row r="72" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="109"/>
+      <c r="B72" s="109"/>
+      <c r="C72" s="109"/>
+      <c r="D72" s="109"/>
+      <c r="E72" s="109"/>
+      <c r="F72" s="109"/>
+      <c r="G72" s="109"/>
+      <c r="H72" s="109"/>
+    </row>
+    <row r="73" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="109"/>
+      <c r="B73" s="109"/>
+      <c r="C73" s="109"/>
+      <c r="D73" s="109"/>
+      <c r="E73" s="109"/>
+      <c r="F73" s="109"/>
+      <c r="G73" s="109"/>
+      <c r="H73" s="109"/>
+    </row>
+    <row r="74" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="109"/>
+      <c r="B74" s="109"/>
+      <c r="C74" s="109"/>
+      <c r="D74" s="109"/>
+      <c r="E74" s="109"/>
+      <c r="F74" s="109"/>
+      <c r="G74" s="109"/>
+      <c r="H74" s="109"/>
+    </row>
+    <row r="75" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="109"/>
+      <c r="B75" s="109"/>
+      <c r="C75" s="109"/>
+      <c r="D75" s="109"/>
+      <c r="E75" s="109"/>
+      <c r="F75" s="109"/>
+      <c r="G75" s="109"/>
+      <c r="H75" s="109"/>
+    </row>
+    <row r="76" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="109"/>
+      <c r="B76" s="109"/>
+      <c r="C76" s="109"/>
+      <c r="D76" s="109"/>
+      <c r="E76" s="109"/>
+      <c r="F76" s="109"/>
+      <c r="G76" s="109"/>
+      <c r="H76" s="109"/>
+    </row>
+    <row r="77" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="109"/>
+      <c r="B77" s="109"/>
+      <c r="C77" s="109"/>
+      <c r="D77" s="109"/>
+      <c r="E77" s="109"/>
+      <c r="F77" s="109"/>
+      <c r="G77" s="109"/>
+      <c r="H77" s="109"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="58">
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="F34:H34"/>
@@ -2767,18 +2741,49 @@
     <mergeCell ref="D36:E36"/>
     <mergeCell ref="F36:H36"/>
     <mergeCell ref="B44:E44"/>
-    <mergeCell ref="A52:H52"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="D37:E37"/>
     <mergeCell ref="F37:H37"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="C38:H38"/>
-    <mergeCell ref="B48:G49"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="C49:F49"/>
     <mergeCell ref="A51:H51"/>
-    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A69:H69"/>
+    <mergeCell ref="A70:H70"/>
+    <mergeCell ref="A71:H71"/>
+    <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A74:H74"/>
+    <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A76:H76"/>
+    <mergeCell ref="A77:H77"/>
   </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="96" orientation="portrait" r:id="rId1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="46" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>